<commit_message>
Atualizando data/season_2025/next_games/next_games.xlsx via script
</commit_message>
<xml_diff>
--- a/data/season_2025/next_games/next_games.xlsx
+++ b/data/season_2025/next_games/next_games.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S54"/>
+  <dimension ref="A1:S51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -526,68 +526,68 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Liga Profesional de Fútbol - ARG PD</t>
+          <t>La Liga 2 - ESP S</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Argentinos Juniors vs Lanús</t>
+          <t>SD Eibar vs Las Palmas</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-03-27 00:00:00</t>
+          <t>2026-03-29 12:00:00</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2.05</t>
+          <t>2.30</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2.80</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>4.75</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>2.52</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2.88</t>
+          <t>2.95</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>4.72</t>
+          <t>3.29</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.66</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.10</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>1.69</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2.40</t>
+          <t>2.17</t>
         </is>
       </c>
       <c r="O2" t="inlineStr"/>
@@ -603,50 +603,70 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>J1 100 Year Vision League - J1-100</t>
+          <t>Primera Division - URY CL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Vissel Kobe vs Sanfrecce Hiroshima</t>
+          <t>Atlético Progreso vs Liverpool</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-03-27 10:00:00</t>
+          <t>2026-03-29 13:00:00</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2.50</t>
+          <t>3.75</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>3.30</t>
+          <t>3.10</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2.80</t>
+          <t>1.90</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>3.73</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>3.34</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2.06</t>
+        </is>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1.95</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+          <t>1.90</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1.83</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>1.93</t>
+        </is>
+      </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
@@ -661,189 +681,213 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Córdoba vs Mirandés</t>
+          <t>Cultural Leonesa vs FC Andorra</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-03-27 18:00:00</t>
+          <t>2026-03-29 14:15:00</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>2.37</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>3.80</t>
+          <t>3.20</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>5.00</t>
+          <t>2.90</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1.66</t>
+          <t>2.51</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>3.84</t>
+          <t>3.29</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>5.52</t>
+          <t>3.03</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>1.83</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1.66</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2.23</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>1.68</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
+          <t>1.83</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>1.85</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>1.95</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2.04</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1.85</t>
+        </is>
+      </c>
       <c r="S4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Liga BetPlay - COL PA</t>
+          <t>Liga Portugal 2 - PRT SL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Rionegro Águilas vs Alianza Petrolera</t>
+          <t>União de Leiria vs Paços de Ferreira</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-03-27 21:00:00</t>
+          <t>2026-03-29 14:30:00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>1.70</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>3.00</t>
+          <t>3.30</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3.90</t>
+          <t>4.50</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2.13</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2.94</t>
+          <t>3.71</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>4.07</t>
+          <t>4.54</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>1.90</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2.20</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>1.85</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2.30</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+          <t>1.95</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>1.87</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>1.92</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1.87</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>1.95</t>
+        </is>
+      </c>
       <c r="S5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Liga BetPlay - COL PA</t>
+          <t>Primera Division - URY CL</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Atlético Bucaramanga vs Santa Fe</t>
+          <t>Juventud vs Boston River</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-03-28 01:10:00</t>
+          <t>2026-03-29 16:00:00</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.95</t>
+          <t>2.20</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>3.30</t>
+          <t>3.10</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>4.20</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1.98</t>
+          <t>2.32</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3.15</t>
+          <t>3.17</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>4.27</t>
+          <t>3.19</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -858,12 +902,12 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>1.68</t>
+          <t>1.71</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2.16</t>
+          <t>2.07</t>
         </is>
       </c>
       <c r="O6" t="inlineStr"/>
@@ -875,83 +919,159 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>J1 100 Year Vision League - J1-100</t>
+          <t>La Liga 2 - ESP S</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Machida Zelvia vs Kawasaki Frontale</t>
+          <t>Real Zaragoza vs Racing Santander</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-03-28 05:00:00</t>
+          <t>2026-03-29 16:30:00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.95</t>
+          <t>2.60</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3.60</t>
+          <t>3.30</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3.60</t>
+          <t>2.70</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2.92</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>3.28</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2.49</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>2.00</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1.66</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
+          <t>1.72</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2.21</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>1.97</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>1.82</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>2.02</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1.86</t>
+        </is>
+      </c>
       <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>La Liga 2 - ESP S</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Nara Club vs Zweigen Kanazawa</t>
+          <t>Almería vs Real Sociedad II</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-03-28 05:00:00</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
+          <t>2026-03-29 19:00:00</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1.53</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>4.10</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>5.50</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>4.12</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>6.14</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1.66</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2.14</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>1.71</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
@@ -961,30 +1081,70 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>Primera Division - URY CL</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Gifu vs Parceiro Nagano</t>
+          <t>Defensor Sporting vs Albion</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-03-28 05:00:00</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+          <t>2026-03-29 19:00:00</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2.05</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2.90</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>3.40</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2.17</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>3.04</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>3.69</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>1.66</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>1.70</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
@@ -994,32 +1154,80 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>Liga BetPlay - COL PA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fujieda MYFC vs Consadole Sapporo</t>
+          <t>Internacional de Bogotá vs Junior FC</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-03-28 05:00:00</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
+          <t>2026-03-29 21:10:00</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2.55</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2.80</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2.61</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>3.19</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>1.72</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2.01</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>1.76</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>2.02</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1.77</t>
+        </is>
+      </c>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
@@ -1027,61 +1235,137 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>Serie A - BRA CB</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Ventforet Kofu vs Omiya Ardija</t>
+          <t>Athletico PR vs Botafogo</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-03-28 05:00:00</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+          <t>2026-03-29 22:30:00</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>4.00</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1.96</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>3.39</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>4.10</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>1.90</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>1.90</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>2.03</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1.81</t>
+        </is>
+      </c>
       <c r="S11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>Primera Division - URY CL</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yokohama vs Shonan Bellmare</t>
+          <t>Peñarol vs Racing</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-03-28 05:00:00</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+          <t>2026-03-29 22:30:00</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1.57</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>3.40</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>5.50</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1.62</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>6.92</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>1.61</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2.20</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
@@ -1093,176 +1377,224 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>Liga BetPlay - COL PA</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ThespaKusatsu Gunma vs Tochigi</t>
+          <t>Deportivo Pasto vs Atlético Nacional</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-03-28 05:00:00</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
+          <t>2026-03-29 23:20:00</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2.25</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>3.37</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>3.11</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2.25</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>1.90</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>1.99</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>1.83</t>
+        </is>
+      </c>
       <c r="S13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>K League 1 - KOR KL</t>
+          <t>Liga BetPlay - COL PA</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pohang Steelers vs Gangwon</t>
+          <t>Llaneros vs Once Caldas</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-03-28 06:00:00</t>
+          <t>2026-03-30 01:30:00</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2.87</t>
+          <t>2.70</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2.90</t>
+          <t>3.40</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2.50</t>
+          <t>2.45</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>3.01</t>
+          <t>2.89</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2.95</t>
+          <t>3.03</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2.64</t>
+          <t>2.61</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1.66</t>
+          <t>2.20</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>1.61</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.95</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2.13</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
+          <t>1.81</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>1.81</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>2.01</t>
+        </is>
+      </c>
       <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>La Liga 2 - ESP S</t>
+          <t>Primera Division - URY CL</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ceuta vs Cádiz</t>
+          <t>Cerro Largo vs Danubio</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-03-28 13:00:00</t>
+          <t>2026-03-30 21:00:00</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>3.20</t>
+          <t>2.90</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3.20</t>
+          <t>2.37</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2.24</t>
+          <t>3.09</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>3.29</t>
+          <t>3.07</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>3.35</t>
+          <t>2.42</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>1.90</t>
+          <t>1.72</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
           <t>2.00</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>1.83</t>
-        </is>
-      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
@@ -1272,70 +1604,62 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>La Liga 2 - ESP S</t>
+          <t>Liga BetPlay - COL PA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Granada vs Huesca</t>
+          <t>Independiente Medellín vs América de Cali</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-03-28 15:15:00</t>
+          <t>2026-03-30 23:10:00</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>2.10</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>3.30</t>
+          <t>3.20</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>4.75</t>
+          <t>3.70</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1.79</t>
+          <t>2.19</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>3.42</t>
+          <t>3.12</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>4.95</t>
+          <t>3.51</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>1.83</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2.20</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>1.64</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>2.25</t>
-        </is>
-      </c>
+          <t>1.83</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
@@ -1345,48 +1669,48 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>La Liga 2 - ESP S</t>
+          <t>Primera Division - URY CL</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Real Valladolid vs Burgos</t>
+          <t>Central Español vs Deportivo Maldonado</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-03-28 15:15:00</t>
+          <t>2026-03-31 00:00:00</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2.15</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>3.10</t>
+          <t>2.90</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>3.50</t>
+          <t>2.25</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2.20</t>
+          <t>3.36</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>3.11</t>
+          <t>2.84</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>3.63</t>
+          <t>2.43</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1399,16 +1723,8 @@
           <t>2.10</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>1.69</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>2.17</t>
-        </is>
-      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
@@ -1418,206 +1734,210 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>La Liga 2 - ESP S</t>
+          <t>Liga BetPlay - COL PA</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Málaga vs Leganés</t>
+          <t>Millonarios vs Fortaleza CEIF</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-03-28 17:30:00</t>
+          <t>2026-03-31 01:20:00</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2.00</t>
+          <t>1.53</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>3.30</t>
+          <t>3.90</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>3.70</t>
+          <t>6.50</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2.06</t>
+          <t>1.52</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>3.31</t>
+          <t>3.93</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>3.80</t>
+          <t>6.47</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.83</t>
+          <t>1.66</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1.83</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>1.90</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>1.90</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>2.02</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>1.77</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
       <c r="S18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Primera Division - URY CL</t>
+          <t>La Liga 2 - ESP S</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Wanderers vs Cerro</t>
+          <t>Mirandés vs Albacete</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-03-28 19:00:00</t>
+          <t>2026-03-31 17:00:00</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>2.60</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2.87</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.40</t>
+          <t>2.70</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2.18</t>
+          <t>2.64</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>3.02</t>
+          <t>3.26</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>3.67</t>
+          <t>2.77</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>2.00</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2.20</t>
+          <t>1.72</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>2.01</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>1.83</t>
+        </is>
+      </c>
       <c r="S19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>La Liga 2 - ESP S</t>
+          <t>Liga Profesional de Fútbol - ARG PD</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Albacete vs Castellón</t>
+          <t>Aldosivi vs Argentinos Juniors</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-03-28 20:00:00</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>2.70</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>3.50</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>2.50</t>
-        </is>
-      </c>
+          <t>2026-03-31 17:00:00</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2.74</t>
+          <t>4.45</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>3.47</t>
+          <t>3.14</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2.53</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>2.25</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>1.57</t>
-        </is>
-      </c>
+          <t>1.96</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
-          <t>2.37</t>
+          <t>1.62</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>1.58</t>
+          <t>2.29</t>
         </is>
       </c>
       <c r="O20" t="inlineStr"/>
@@ -1634,171 +1954,183 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Sporting Gijón vs Deportivo La Coruña</t>
+          <t>Deportivo La Coruña vs Córdoba</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-03-28 20:00:00</t>
+          <t>2026-03-31 18:00:00</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2.35</t>
+          <t>1.95</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>3.10</t>
+          <t>3.60</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>3.00</t>
+          <t>3.80</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2.60</t>
+          <t>1.94</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2.95</t>
+          <t>3.65</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>3.08</t>
+          <t>3.81</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>1.83</t>
+          <t>2.00</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>1.83</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>1.92</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>1.88</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
+          <t>1.72</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>1.82</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>1.97</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>1.84</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
       <c r="S21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Liga BetPlay - COL PA</t>
+          <t>La Liga 2 - ESP S</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Cúcuta Deportivo vs Boyacá Chicó</t>
+          <t>Real Valladolid vs Cádiz</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-03-28 21:00:00</t>
+          <t>2026-03-31 19:30:00</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>1.72</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>3.50</t>
+          <t>3.70</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>5.75</t>
+          <t>4.75</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1.64</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>3.63</t>
+          <t>3.67</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>5.56</t>
+          <t>4.84</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>1.66</t>
+          <t>1.83</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>1.83</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>2.02</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>1.77</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>2.04</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
       <c r="S22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Primera Division - URY CL</t>
+          <t>Liga BetPlay - COL PA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Montevideo City Torque vs Nacional</t>
+          <t>Deportes Tolima vs Rionegro Águilas</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-03-28 22:30:00</t>
+          <t>2026-04-01 01:00:00</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>3.42</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>3.24</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>2.17</t>
-        </is>
-      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
@@ -1812,60 +2144,28 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Liga BetPlay - COL PA</t>
+          <t>J1 100 Year Vision League - J1-100</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Deportes Tolima vs Jaguares de Córdoba</t>
+          <t>Vissel Kobe vs Shimizu S-Pulse</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-03-28 23:10:00</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>1.38</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>4.33</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>9.50</t>
-        </is>
-      </c>
+          <t>2026-04-01 10:00:00</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>1.34</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>4.42</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>10.00</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>1.50</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>2.50</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
@@ -1877,106 +2177,50 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Liga BetPlay - COL PA</t>
+          <t>J1 100 Year Vision League - J1-100</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Deportivo Cali vs Deportivo Pereira</t>
+          <t>Machida Zelvia vs FC Tokyo</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-03-29 01:20:00</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>1.44</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>3.80</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>9.50</t>
-        </is>
-      </c>
+          <t>2026-04-01 10:00:00</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>1.39</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>4.05</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>9.54</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>1.40</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>2.75</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>1.44</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>2.71</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>1.90</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>1.90</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>2.02</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>1.78</t>
-        </is>
-      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>La Liga 2 - ESP S</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Roasso Kumamoto vs Kagoshima United</t>
+          <t>FC Andorra vs Málaga</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-03-29 04:00:00</t>
+          <t>2026-04-01 17:00:00</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -1999,28 +2243,60 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>La Liga 2 - ESP S</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Vanraure Hachinohe vs Sagamihara</t>
+          <t>Burgos vs Ceuta</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-03-29 04:00:00</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
+          <t>2026-04-01 18:00:00</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>5.00</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>1.81</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>3.38</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>4.87</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>1.61</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2.20</t>
+        </is>
+      </c>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
@@ -2032,17 +2308,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>La Liga 2 - ESP S</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Giravanz Kitakyushu vs Ryūkyū</t>
+          <t>Huesca vs Cultural Leonesa</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-03-29 05:00:00</t>
+          <t>2026-04-01 18:00:00</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -2065,17 +2341,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>La Liga 2 - ESP S</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Renofa Yamaguchi vs Oita Trinita</t>
+          <t>Racing Santander vs Sporting Gijón</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-03-29 05:00:00</t>
+          <t>2026-04-01 19:30:00</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -2098,17 +2374,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>Liga BetPlay - COL PA</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Gainare Tottori vs Sagan Tosu</t>
+          <t>Alianza Petrolera vs Deportivo Pasto</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-03-29 05:00:00</t>
+          <t>2026-04-01 21:10:00</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -2131,28 +2407,60 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>Serie A - BRA CB</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Rayluck Shiga vs Tegevajaro Miyazaki</t>
+          <t>Internacional vs São Paulo</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-03-29 05:00:00</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
+          <t>2026-04-01 22:30:00</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2.20</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>3.30</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2.92</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>3.78</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>1.90</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>1.90</t>
+        </is>
+      </c>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
@@ -2164,28 +2472,48 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>Serie A - BRA CB</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Tokushima Vortis vs Kochi United</t>
+          <t>Botafogo vs Mirassol</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-03-29 05:00:00</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
+          <t>2026-04-01 22:30:00</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>3.60</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>1.95</t>
+        </is>
+      </c>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
@@ -2197,28 +2525,48 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>Serie A - BRA CB</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Kamatamare Sanuki vs Ehime</t>
+          <t>Bahia vs Athletico PR</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-03-29 05:00:00</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
+          <t>2026-04-01 23:00:00</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>1.90</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>3.40</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>4.10</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>1.95</t>
+        </is>
+      </c>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
@@ -2230,28 +2578,60 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>Serie A - BRA CB</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Osaka vs Albirex Niigata</t>
+          <t>Cruzeiro vs Vitória</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-03-29 05:00:00</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
+          <t>2026-04-01 23:00:00</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>1.55</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>3.70</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>6.00</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>1.59</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>3.83</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>6.17</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>1.66</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr"/>
       <c r="O34" t="inlineStr"/>
@@ -2263,26 +2643,38 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>Liga Profesional de Fútbol - ARG PD</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Kataller Toyama vs Imabari</t>
+          <t>Lanús vs Platense</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-03-29 05:00:00</t>
+          <t>2026-04-01 23:00:00</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>1.94</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>3.15</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>4.54</t>
+        </is>
+      </c>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
@@ -2296,28 +2688,60 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>Serie A - BRA CB</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Iwaki vs Júbilo Iwata</t>
+          <t>Coritiba vs Vasco da Gama</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-03-29 05:00:00</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
+          <t>2026-04-01 23:30:00</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2.50</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2.80</t>
+        </is>
+      </c>
       <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2.58</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>3.13</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2.94</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>1.95</t>
+        </is>
+      </c>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
@@ -2329,17 +2753,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>Liga BetPlay - COL PA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Fukushima United vs Matsumoto Yamaga</t>
+          <t>Santa Fe vs Llaneros</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-03-29 05:00:00</t>
+          <t>2026-04-01 23:30:00</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -2362,28 +2786,60 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>Serie A - BRA CB</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Montedio Yamagata vs Tochigi City</t>
+          <t>Fluminense vs Corinthians</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-03-29 05:00:00</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
+          <t>2026-04-02 00:30:00</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>1.90</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>4.33</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>1.91</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>3.32</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>4.42</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>1.70</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2.05</t>
+        </is>
+      </c>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
@@ -2395,17 +2851,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>J2/J3 100 Year Vision League - None</t>
+          <t>Liga BetPlay - COL PA</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Blaublitz Akita vs Vegalta Sendai</t>
+          <t>Atlético Nacional vs Cúcuta Deportivo</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-03-29 05:00:00</t>
+          <t>2026-04-02 01:30:00</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2433,65 +2889,25 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SD Eibar vs Las Palmas</t>
+          <t>Las Palmas vs Granada</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-03-29 12:00:00</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>2.40</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>2.90</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
-      </c>
+          <t>2026-04-02 17:00:00</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>2.50</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>2.91</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>3.28</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>1.61</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>2.20</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>1.69</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>2.17</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
@@ -2501,70 +2917,30 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Primera Division - URY CL</t>
+          <t>La Liga 2 - ESP S</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Atlético Progreso vs Liverpool</t>
+          <t>Castellón vs Almería</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-03-29 13:00:00</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>3.60</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>1.95</t>
-        </is>
-      </c>
+          <t>2026-04-02 18:00:00</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>3.69</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>3.30</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>2.04</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>1.83</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>1.83</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>1.83</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>1.93</t>
-        </is>
-      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
@@ -2579,235 +2955,135 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Cultural Leonesa vs FC Andorra</t>
+          <t>Real Sociedad II vs SD Eibar</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-03-29 14:15:00</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>2.45</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>3.30</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>2.75</t>
-        </is>
-      </c>
+          <t>2026-04-02 18:00:00</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>2.50</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>3.35</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>2.85</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>1.90</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>2.00</t>
-        </is>
-      </c>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>2.06</t>
-        </is>
-      </c>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>1.79</t>
-        </is>
-      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Liga Portugal 2 - PRT SL</t>
+          <t>Liga Profesional de Fútbol - ARG PD</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>União de Leiria vs Paços de Ferreira</t>
+          <t>Barracas Central vs Sarmiento</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-03-29 14:30:00</t>
+          <t>2026-04-02 18:00:00</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>1.70</t>
+          <t>2.35</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>3.30</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>4.50</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1.76</t>
+          <t>2.35</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>3.67</t>
+          <t>2.90</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>4.48</t>
+          <t>3.58</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>1.90</t>
+          <t>1.53</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>1.85</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>1.95</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>1.90</t>
-        </is>
-      </c>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t>1.90</t>
-        </is>
-      </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>1.86</t>
-        </is>
-      </c>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>1.91</t>
-        </is>
-      </c>
+          <t>2.37</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Primera Division - URY CL</t>
+          <t>Liga BetPlay - COL PA</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Juventud vs Boston River</t>
+          <t>Boyacá Chicó vs Deportivo Pereira</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-03-29 16:00:00</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>2.30</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>2.80</t>
-        </is>
-      </c>
+          <t>2026-04-02 19:00:00</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
-          <t>2.44</t>
+          <t>2.09</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>3.14</t>
+          <t>3.21</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>3.01</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>1.66</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>1.71</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>2.07</t>
-        </is>
-      </c>
+          <t>3.68</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
@@ -2822,154 +3098,70 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Real Zaragoza vs Racing Santander</t>
+          <t>Leganés vs Real Zaragoza</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-03-29 16:30:00</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>2.75</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>3.30</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>2.40</t>
-        </is>
-      </c>
+          <t>2026-04-02 19:30:00</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>3.13</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>2.97</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>2.55</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>2.00</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>1.72</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>2.21</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>1.67</t>
-        </is>
-      </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>2.00</t>
-        </is>
-      </c>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>2.00</t>
-        </is>
-      </c>
-      <c r="R45" t="inlineStr">
-        <is>
-          <t>1.84</t>
-        </is>
-      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>La Liga 2 - ESP S</t>
+          <t>Liga Profesional de Fútbol - ARG PD</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Almería vs Real Sociedad II</t>
+          <t>Tigre vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-03-29 19:00:00</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>1.55</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>4.00</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>5.50</t>
-        </is>
-      </c>
+          <t>2026-04-02 20:30:00</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1.53</t>
+          <t>2.27</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>4.16</t>
+          <t>2.88</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>6.19</t>
-        </is>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>2.00</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>1.72</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>2.14</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>1.71</t>
-        </is>
-      </c>
+          <t>3.81</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr"/>
@@ -2979,70 +3171,30 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Primera Division - URY CL</t>
+          <t>Liga BetPlay - COL PA</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Defensor Sporting vs Albion</t>
+          <t>América de Cali vs Atlético Bucaramanga</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-03-29 19:00:00</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>2.05</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>2.90</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>3.40</t>
-        </is>
-      </c>
+          <t>2026-04-02 21:10:00</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>2.17</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>3.04</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>3.69</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>1.66</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>1.69</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>2.12</t>
-        </is>
-      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
       <c r="Q47" t="inlineStr"/>
@@ -3052,40 +3204,60 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Liga BetPlay - COL PA</t>
+          <t>Serie A - BRA CB</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Internacional de Bogotá vs Junior FC</t>
+          <t>Chapecoense vs Atlético Mineiro</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-03-29 21:10:00</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
+          <t>2026-04-02 22:00:00</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2.87</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2.45</t>
+        </is>
+      </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
-          <t>2.91</t>
+          <t>2.87</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>3.40</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2.43</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
+          <t>2.47</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>1.90</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>1.90</t>
+        </is>
+      </c>
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr"/>
@@ -3102,71 +3274,47 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Athletico PR vs Botafogo</t>
+          <t>Santos vs Remo</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-03-29 22:30:00</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>2.00</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>3.20</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>4.00</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
-      </c>
+          <t>2026-04-02 22:00:00</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>1.52</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>3.40</t>
+          <t>4.18</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>3.87</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>1.90</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>1.90</t>
-        </is>
-      </c>
+          <t>6.47</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr"/>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>2.03</t>
+          <t>1.85</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.98</t>
         </is>
       </c>
       <c r="S49" t="inlineStr"/>
@@ -3174,60 +3322,28 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Primera Division - URY CL</t>
+          <t>Liga BetPlay - COL PA</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Peñarol vs Racing</t>
+          <t>Jaguares de Córdoba vs Millonarios</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-03-29 22:30:00</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>1.65</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>3.25</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>5.00</t>
-        </is>
-      </c>
+          <t>2026-04-02 23:20:00</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>1.71</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>3.07</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>6.28</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>1.66</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr"/>
@@ -3239,17 +3355,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Liga BetPlay - COL PA</t>
+          <t>Liga Profesional de Fútbol - ARG PD</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Deportivo Pasto vs Atlético Nacional</t>
+          <t>Talleres Córdoba vs Boca Juniors</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-03-29 23:20:00</t>
+          <t>2026-04-02 23:30:00</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -3258,17 +3374,17 @@
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
-          <t>3.45</t>
+          <t>2.97</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>3.05</t>
+          <t>2.84</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.77</t>
         </is>
       </c>
       <c r="K51" t="inlineStr"/>
@@ -3281,217 +3397,6 @@
       <c r="R51" t="inlineStr"/>
       <c r="S51" t="inlineStr"/>
     </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Liga BetPlay - COL PA</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Llaneros vs Once Caldas</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>2026-03-30 01:30:00</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>2.62</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>3.20</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>2.55</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>2.89</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>3.02</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>2.61</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>1.83</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>1.83</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>1.95</t>
-        </is>
-      </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>1.81</t>
-        </is>
-      </c>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr">
-        <is>
-          <t>2.02</t>
-        </is>
-      </c>
-      <c r="R52" t="inlineStr">
-        <is>
-          <t>1.78</t>
-        </is>
-      </c>
-      <c r="S52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Primera Division - URY CL</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Cerro Largo vs Danubio</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>2026-03-30 21:00:00</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>2.87</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>2.90</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>2.30</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>3.09</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>3.07</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>2.42</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>1.66</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
-      <c r="R53" t="inlineStr"/>
-      <c r="S53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Liga BetPlay - COL PA</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Independiente Medellín vs América de Cali</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>2026-03-30 23:10:00</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>1.95</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>3.25</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>3.70</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>2.03</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>3.22</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>3.87</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>1.83</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>1.83</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
-      <c r="R54" t="inlineStr"/>
-      <c r="S54" t="inlineStr"/>
-    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S2" r:id="rId1"/>

</xml_diff>